<commit_message>
su data 2025 processed
</commit_message>
<xml_diff>
--- a/data/su/original_data/bpc_su_2025.xlsx
+++ b/data/su/original_data/bpc_su_2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="U:\OA\Open APC Sweden - Filer till KB\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C98487F4-9458-4490-96A3-2CCF228A9780}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8CDE7CBC-EFA6-4B29-84DD-5780B8A833AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7155" yWindow="3915" windowWidth="25125" windowHeight="15285" xr2:uid="{D9C9CFD0-73BD-A64C-9F3E-974AFC89DE91}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{D9C9CFD0-73BD-A64C-9F3E-974AFC89DE91}"/>
   </bookViews>
   <sheets>
     <sheet name="Blad1" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="53">
   <si>
     <t>institution</t>
   </si>
@@ -604,18 +604,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3E71BB5E-CB6D-AB41-AAD4-1BB745BAAAAD}">
-  <dimension ref="A1:J18"/>
-  <sheetFormatPr defaultColWidth="11.109375" defaultRowHeight="15"/>
+  <dimension ref="A1:J16"/>
+  <sheetFormatPr defaultColWidth="11.07421875" defaultRowHeight="15.5"/>
   <cols>
-    <col min="1" max="1" width="51.44140625" customWidth="1"/>
-    <col min="2" max="3" width="10.6640625" customWidth="1"/>
-    <col min="4" max="4" width="22.88671875" customWidth="1"/>
-    <col min="5" max="5" width="13.44140625" customWidth="1"/>
-    <col min="6" max="6" width="28.5546875" customWidth="1"/>
-    <col min="7" max="7" width="48.5546875" customWidth="1"/>
-    <col min="8" max="8" width="18.44140625" style="4" customWidth="1"/>
+    <col min="1" max="1" width="51.4609375" customWidth="1"/>
+    <col min="2" max="3" width="10.69140625" customWidth="1"/>
+    <col min="4" max="4" width="22.84375" customWidth="1"/>
+    <col min="5" max="5" width="13.4609375" customWidth="1"/>
+    <col min="6" max="6" width="28.53515625" customWidth="1"/>
+    <col min="7" max="7" width="48.53515625" customWidth="1"/>
+    <col min="8" max="8" width="18.4609375" style="4" customWidth="1"/>
     <col min="9" max="9" width="13" customWidth="1"/>
-    <col min="10" max="10" width="12.5546875" customWidth="1"/>
+    <col min="10" max="10" width="12.53515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="18">
@@ -825,7 +825,7 @@
         <v>2025</v>
       </c>
       <c r="C9">
-        <v>38761.660000000003</v>
+        <v>115315.67</v>
       </c>
       <c r="D9" t="s">
         <v>24</v>
@@ -842,25 +842,25 @@
     </row>
     <row r="10" spans="1:10">
       <c r="A10" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="B10">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="C10">
-        <v>30000</v>
+        <v>40614.120000000003</v>
       </c>
       <c r="D10" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="F10" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="G10" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:10">
@@ -868,45 +868,48 @@
         <v>30</v>
       </c>
       <c r="B11">
-        <v>2025</v>
-      </c>
-      <c r="C11">
-        <v>46554.01</v>
+        <v>2026</v>
+      </c>
+      <c r="C11" s="2">
+        <v>116040.33</v>
       </c>
       <c r="D11" t="s">
-        <v>24</v>
+        <v>52</v>
       </c>
       <c r="E11" t="s">
         <v>45</v>
       </c>
       <c r="F11" t="s">
-        <v>13</v>
+        <v>47</v>
       </c>
       <c r="G11" t="s">
-        <v>37</v>
+        <v>39</v>
+      </c>
+      <c r="H11" s="4">
+        <v>9781529257687</v>
       </c>
     </row>
     <row r="12" spans="1:10">
       <c r="A12" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="B12">
-        <v>2024</v>
-      </c>
-      <c r="C12">
-        <v>40614.120000000003</v>
+        <v>2025</v>
+      </c>
+      <c r="C12" s="2">
+        <v>70784.600000000006</v>
       </c>
       <c r="D12" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="E12" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="F12" t="s">
-        <v>17</v>
+        <v>13</v>
       </c>
       <c r="G12" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:10">
@@ -917,45 +920,42 @@
         <v>2026</v>
       </c>
       <c r="C13" s="2">
-        <v>116040.33</v>
+        <v>77360.22</v>
       </c>
       <c r="D13" t="s">
-        <v>52</v>
+        <v>27</v>
       </c>
       <c r="E13" t="s">
         <v>45</v>
       </c>
       <c r="F13" t="s">
-        <v>47</v>
+        <v>15</v>
       </c>
       <c r="G13" t="s">
-        <v>39</v>
-      </c>
-      <c r="H13" s="4">
-        <v>9781529257687</v>
+        <v>41</v>
       </c>
     </row>
     <row r="14" spans="1:10">
       <c r="A14" t="s">
-        <v>30</v>
+        <v>50</v>
       </c>
       <c r="B14">
-        <v>2025</v>
+        <v>2026</v>
       </c>
       <c r="C14" s="2">
-        <v>70784.600000000006</v>
+        <v>34453.61</v>
       </c>
       <c r="D14" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E14" t="s">
         <v>45</v>
       </c>
       <c r="F14" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="G14" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15" spans="1:10">
@@ -966,90 +966,44 @@
         <v>2026</v>
       </c>
       <c r="C15" s="2">
-        <v>77360.22</v>
+        <v>111002.6</v>
       </c>
       <c r="D15" t="s">
-        <v>27</v>
+        <v>46</v>
       </c>
       <c r="E15" t="s">
         <v>45</v>
       </c>
       <c r="F15" t="s">
-        <v>15</v>
-      </c>
-      <c r="G15" t="s">
-        <v>41</v>
+        <v>17</v>
+      </c>
+      <c r="G15" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H15" s="4">
+        <v>9781003699408</v>
       </c>
     </row>
     <row r="16" spans="1:10">
       <c r="A16" t="s">
-        <v>50</v>
+        <v>30</v>
       </c>
       <c r="B16">
-        <v>2026</v>
+        <v>2025</v>
       </c>
       <c r="C16" s="2">
-        <v>34453.61</v>
+        <v>134584.70000000001</v>
       </c>
       <c r="D16" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="E16" t="s">
         <v>45</v>
       </c>
       <c r="F16" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G16" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8">
-      <c r="A17" t="s">
-        <v>30</v>
-      </c>
-      <c r="B17">
-        <v>2026</v>
-      </c>
-      <c r="C17" s="2">
-        <v>111002.6</v>
-      </c>
-      <c r="D17" t="s">
-        <v>46</v>
-      </c>
-      <c r="E17" t="s">
-        <v>45</v>
-      </c>
-      <c r="F17" t="s">
-        <v>17</v>
-      </c>
-      <c r="G17" s="6" t="s">
-        <v>51</v>
-      </c>
-      <c r="H17" s="4">
-        <v>9781003699408</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8">
-      <c r="A18" t="s">
-        <v>30</v>
-      </c>
-      <c r="B18">
-        <v>2025</v>
-      </c>
-      <c r="C18" s="2">
-        <v>134584.70000000001</v>
-      </c>
-      <c r="D18" t="s">
-        <v>29</v>
-      </c>
-      <c r="E18" t="s">
-        <v>45</v>
-      </c>
-      <c r="F18" t="s">
-        <v>15</v>
-      </c>
-      <c r="G18" t="s">
         <v>43</v>
       </c>
     </row>

</xml_diff>